<commit_message>
fix minor issues in P2
</commit_message>
<xml_diff>
--- a/P2/CS795_Retrieval_Results.xlsx
+++ b/P2/CS795_Retrieval_Results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,14 +509,14 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> What are the limitation of previous works on MCP servers</t>
+          <t>What is MCP client?</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>0.52</v>
+        <v>0.5834</v>
       </c>
       <c r="D5" t="n">
         <v>10</v>
@@ -530,56 +530,56 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> What are the limitation of previous works on MCP servers</t>
+          <t>What is MCP client?</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>2</v>
       </c>
       <c r="C6" t="n">
-        <v>0.4776</v>
+        <v>0.5562</v>
       </c>
       <c r="D6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>and permission scope within the MCP architecture. #### MCP Server / Tool Execution The MCP Server / Tool Execution layer represents the runtime environment in which MCP tools are implemented and executed, including server-side logic, exposed APIs, authentication checks, plugin loading, and resource management. This layer is responsible for safely handling inputs received from MCP hosts and clients, enforcing isolation boundaries, and ensuring that tool execution does not violate system or data integrity. Security failures here typically arise from unsafe execution environments, weak authentication or authorization, overly permissive introspection interfaces, or inadequate isolation between tools and underlying infrastructure. Because this</t>
+          <t>control point prior to tool invocation. #### MCP Client / SDK The MCP Client / SDK layer comprises the software runtime that bridges the language model–driven agent with external MCP servers, handling protocol parsing, request construction, response interpretation, and local execution logic. This layer operates at a sensitive trust boundary, as it transforms high-level model decisions into concrete network interactions and local actions, often within proximity to user resources and credentials. Security risks arise when client implementations implicitly trust server responses, fail to enforce strict schemas, or allow model-influenced output to trigger unintended behavior. Because the client mediates both inbound</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> What are the limitation of previous works on MCP servers</t>
+          <t>What is MCP client?</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>3</v>
       </c>
       <c r="C7" t="n">
-        <v>0.4264</v>
+        <v>0.5403</v>
       </c>
       <c r="D7" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>sits upstream of execution and governs how components enter the MCP ecosystem in the first place. Its security role is to ensure authenticity, integrity, and traceability of MCP artifacts before they are ever invoked by a host or client. Failures at this layer undermine trust assumptions across the entire stack: once a malicious or compromised component is registered, updated, or promoted through the supply chain, downstream layers may execute it correctly yet still produce unsafe outcomes. As a result, this layer is fundamental for enforcing trust boundaries, provenance guarantees, and long-term ecosystem safety rather than runtime correctness alone. --- ###</t>
+          <t>layers. Because MCP agents often assume reliable and trustworthy communication, transport-layer compromises can silently subvert otherwise correct behavior at the client, host, or server layers, making robust network-level safeguards essential for preserving end-to-end security guarantees. #### Registry / Marketplace &amp; Supply Chain The Registry / Marketplace – Supply Chain layer captures all mechanisms responsible for discovery, distribution, versioning, and provenance of MCP servers, tools, plugins, and their updates. This layer sits upstream of execution and governs how components enter the MCP ecosystem in the first place. Its security role is to ensure authenticity, integrity, and traceability of MCP artifacts before</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>What are the security best practices for MCP servers?</t>
+          <t xml:space="preserve"> What are the limitation of previous works on MCP servers</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>1</v>
       </c>
       <c r="C8" t="n">
-        <v>0.6577</v>
+        <v>0.52</v>
       </c>
       <c r="D8" t="n">
         <v>10</v>
@@ -593,14 +593,14 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>What are the security best practices for MCP servers?</t>
+          <t xml:space="preserve"> What are the limitation of previous works on MCP servers</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>2</v>
       </c>
       <c r="C9" t="n">
-        <v>0.6056</v>
+        <v>0.4776</v>
       </c>
       <c r="D9" t="n">
         <v>11</v>
@@ -614,19 +614,82 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>What are the security best practices for MCP servers?</t>
+          <t xml:space="preserve"> What are the limitation of previous works on MCP servers</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>3</v>
       </c>
       <c r="C10" t="n">
+        <v>0.4264</v>
+      </c>
+      <c r="D10" t="n">
+        <v>16</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>sits upstream of execution and governs how components enter the MCP ecosystem in the first place. Its security role is to ensure authenticity, integrity, and traceability of MCP artifacts before they are ever invoked by a host or client. Failures at this layer undermine trust assumptions across the entire stack: once a malicious or compromised component is registered, updated, or promoted through the supply chain, downstream layers may execute it correctly yet still produce unsafe outcomes. As a result, this layer is fundamental for enforcing trust boundaries, provenance guarantees, and long-term ecosystem safety rather than runtime correctness alone. --- ###</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>What are the security best practices for MCP servers?</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.6577</v>
+      </c>
+      <c r="D11" t="n">
+        <v>10</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>credentials. Security risks arise when client implementations implicitly trust server responses, fail to enforce strict schemas, or allow model-influenced output to trigger unintended behavior. Because the client mediates both inbound data from servers and outbound actions initiated by the model, weaknesses at this layer can amplify upstream failures or enable direct compromise even when other components behave correctly. Consequently, the client layer is a critical enforcement point for validation, isolation, and permission scope within the MCP architecture. #### MCP Server / Tool Execution The MCP Server / Tool Execution layer represents the runtime environment in which MCP tools are implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>What are the security best practices for MCP servers?</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.6056</v>
+      </c>
+      <c r="D12" t="n">
+        <v>11</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>and permission scope within the MCP architecture. #### MCP Server / Tool Execution The MCP Server / Tool Execution layer represents the runtime environment in which MCP tools are implemented and executed, including server-side logic, exposed APIs, authentication checks, plugin loading, and resource management. This layer is responsible for safely handling inputs received from MCP hosts and clients, enforcing isolation boundaries, and ensuring that tool execution does not violate system or data integrity. Security failures here typically arise from unsafe execution environments, weak authentication or authorization, overly permissive introspection interfaces, or inadequate isolation between tools and underlying infrastructure. Because this</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>What are the security best practices for MCP servers?</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" t="n">
         <v>0.5733</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D13" t="n">
         <v>14</v>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>between authenticated parties, even in the presence of network-level adversaries. Security failures at this layer arise from weak or absent transport protections, such as insufficient authentication of MCP endpoints, lack of message integrity or replay protection, improper session binding, or insecure transport configurations. These weaknesses can enable man-in-the-middle attacks, replay or reordering of tool calls, downgrade attacks, or injection of stale or malicious responses that remain syntactically valid at higher layers. Because MCP agents often assume reliable and trustworthy communication, transport-layer compromises can silently subvert otherwise correct behavior at the client, host, or server layers, making robust network-level safeguards essential</t>
         </is>

</xml_diff>